<commit_message>
reports: refresh canonical surfaces after legacy epithelial backfill
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/comparison_world_biology_summary_v3/comparison_world_biology_summary_v3.xlsx
+++ b/reports/comparison_world_biology_summary_v3/comparison_world_biology_summary_v3.xlsx
@@ -567,7 +567,6 @@
           <t>proximal_anchor</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>organoid (CA1)</t>
@@ -588,8 +587,6 @@
           <t>GSE266789</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="b">
         <v>1</v>
       </c>
@@ -619,11 +616,27 @@
       <c r="P2" t="n">
         <v>88.5</v>
       </c>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>mid_GW14_16</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>week_15</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Basal cells</t>
+        </is>
+      </c>
+      <c r="T2" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="U2" t="n">
+        <v>11.4</v>
+      </c>
       <c r="V2" t="inlineStr">
         <is>
           <t>mixed proximal airway-like epithelial population</t>
@@ -634,7 +647,6 @@
           <t>proximal_anchor</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr"/>
       <c r="Y2" t="inlineStr">
         <is>
           <t>local organoid anchor query</t>
@@ -652,7 +664,6 @@
           <t>proximal_anchor</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>organoid (BU3)</t>
@@ -673,8 +684,6 @@
           <t>GSE266789</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" t="b">
         <v>1</v>
       </c>
@@ -704,11 +713,27 @@
       <c r="P3" t="n">
         <v>98.2</v>
       </c>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>mid_GW14_16</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>week_15</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Basal cells</t>
+        </is>
+      </c>
+      <c r="T3" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="U3" t="n">
+        <v>10.9</v>
+      </c>
       <c r="V3" t="inlineStr">
         <is>
           <t>more converged proximal airway-like epithelial population</t>
@@ -719,7 +744,6 @@
           <t>proximal_anchor</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr"/>
       <c r="Y3" t="inlineStr">
         <is>
           <t>local organoid anchor query</t>
@@ -801,11 +825,27 @@
       <c r="P4" t="n">
         <v>100</v>
       </c>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>late_GW17_19</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>week_18</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Tip cells</t>
+        </is>
+      </c>
+      <c r="T4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U4" t="n">
+        <v>13.3</v>
+      </c>
       <c r="V4" t="inlineStr">
         <is>
           <t>distal late-fetal Tip-like validation</t>
@@ -816,7 +856,6 @@
           <t>donor_resolved_distal</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr"/>
       <c r="Y4" t="inlineStr">
         <is>
           <t>donor-resolved from pooled GSM8229877</t>
@@ -898,11 +937,27 @@
       <c r="P5" t="n">
         <v>100</v>
       </c>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>late_GW17_19</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>week_18</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Tip cells</t>
+        </is>
+      </c>
+      <c r="T5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" t="n">
+        <v>12.6</v>
+      </c>
       <c r="V5" t="inlineStr">
         <is>
           <t>distal late-fetal Tip-like (supportive, low n)</t>
@@ -999,11 +1054,27 @@
       <c r="P6" t="n">
         <v>100</v>
       </c>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>late_GW17_19</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>week_18</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Tip cells</t>
+        </is>
+      </c>
+      <c r="T6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U6" t="n">
+        <v>13.6</v>
+      </c>
       <c r="V6" t="inlineStr">
         <is>
           <t>distal late-fetal Tip-like validation</t>
@@ -1014,7 +1085,6 @@
           <t>donor_resolved_distal</t>
         </is>
       </c>
-      <c r="X6" t="inlineStr"/>
       <c r="Y6" t="inlineStr">
         <is>
           <t>donor-resolved from pooled GSM8229877</t>
@@ -1096,11 +1166,27 @@
       <c r="P7" t="n">
         <v>100</v>
       </c>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>late_GW17_19</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>week_18</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Tip cells</t>
+        </is>
+      </c>
+      <c r="T7" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" t="n">
+        <v>17.1</v>
+      </c>
       <c r="V7" t="inlineStr">
         <is>
           <t>distal late-fetal Tip-like validation</t>
@@ -1111,7 +1197,6 @@
           <t>donor_resolved_distal</t>
         </is>
       </c>
-      <c r="X7" t="inlineStr"/>
       <c r="Y7" t="inlineStr">
         <is>
           <t>donor-resolved from pooled GSM8229877</t>
@@ -1198,7 +1283,6 @@
           <t>late_GW17_19</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr">
         <is>
           <t>Stromal-like cells 1</t>
@@ -1311,7 +1395,6 @@
           <t>late_GW17_19</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr">
         <is>
           <t>Stromal-like cells 1</t>
@@ -1424,7 +1507,6 @@
           <t>late_GW17_19</t>
         </is>
       </c>
-      <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr">
         <is>
           <t>SOX2lowCFTR+ cells</t>
@@ -1446,7 +1528,6 @@
           <t>condition_perturbation</t>
         </is>
       </c>
-      <c r="X10" t="inlineStr"/>
       <c r="Y10" t="inlineStr">
         <is>
           <t>single donor SPC2-ST-B2</t>
@@ -1533,7 +1614,6 @@
           <t>late_GW17_19</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr">
         <is>
           <t>Proliferating progenitors</t>
@@ -1555,7 +1635,6 @@
           <t>differentiation_transitional</t>
         </is>
       </c>
-      <c r="X11" t="inlineStr"/>
       <c r="Y11" t="inlineStr">
         <is>
           <t>condition-level merging 2 biological replicates</t>
@@ -1642,7 +1721,6 @@
           <t>late_GW17_19</t>
         </is>
       </c>
-      <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr">
         <is>
           <t>SOX2lowCFTR+ cells</t>
@@ -1664,7 +1742,6 @@
           <t>differentiation_transitional</t>
         </is>
       </c>
-      <c r="X12" t="inlineStr"/>
       <c r="Y12" t="inlineStr">
         <is>
           <t>condition-level merging 2 biological replicates</t>
@@ -1751,7 +1828,6 @@
           <t>early_GW10_13</t>
         </is>
       </c>
-      <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr">
         <is>
           <t>PNEC</t>
@@ -1773,7 +1849,6 @@
           <t>differentiation_transitional</t>
         </is>
       </c>
-      <c r="X13" t="inlineStr"/>
       <c r="Y13" t="inlineStr">
         <is>
           <t>condition-level merging 2 biological replicates</t>
@@ -1860,7 +1935,6 @@
           <t>early_GW10_13</t>
         </is>
       </c>
-      <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr">
         <is>
           <t>Budtip progenitors</t>
@@ -1947,7 +2021,6 @@
           <t>early_GW10_13</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr">
         <is>
           <t>Epithelial</t>
@@ -1969,7 +2042,6 @@
           <t>early_GW10_13</t>
         </is>
       </c>
-      <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr">
         <is>
           <t>Budtip progenitors</t>
@@ -1991,7 +2063,6 @@
           <t>passage_maturation</t>
         </is>
       </c>
-      <c r="X15" t="inlineStr"/>
       <c r="Y15" t="inlineStr">
         <is>
           <t>GSM-level; citation missing on GEO</t>
@@ -2052,7 +2123,6 @@
           <t>early_GW10_13</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr">
         <is>
           <t>Epithelial</t>
@@ -2074,7 +2144,6 @@
           <t>early_GW10_13</t>
         </is>
       </c>
-      <c r="R16" t="inlineStr"/>
       <c r="S16" t="inlineStr">
         <is>
           <t>Budtip progenitors</t>
@@ -2187,7 +2256,6 @@
           <t>late_GW17_19</t>
         </is>
       </c>
-      <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr">
         <is>
           <t>Proliferating progenitors</t>
@@ -2300,7 +2368,6 @@
           <t>late_GW17_19</t>
         </is>
       </c>
-      <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr">
         <is>
           <t>Proliferating progenitors</t>
@@ -2322,7 +2389,6 @@
           <t>culture_format_comparison</t>
         </is>
       </c>
-      <c r="X18" t="inlineStr"/>
       <c r="Y18" t="inlineStr">
         <is>
           <t>same iPSC line as GSE221343; iAEC2 subset promotion D-0013</t>
@@ -2409,7 +2475,6 @@
           <t>late_GW17_19</t>
         </is>
       </c>
-      <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr">
         <is>
           <t>Proliferating progenitors</t>
@@ -2431,7 +2496,6 @@
           <t>culture_format_comparison</t>
         </is>
       </c>
-      <c r="X19" t="inlineStr"/>
       <c r="Y19" t="inlineStr">
         <is>
           <t>same iPSC line as GSE221343; +MRC5 co-culture; iAEC2 subset promotion D-0013</t>
@@ -2544,7 +2608,6 @@
           <t>perturbation_positive_arm</t>
         </is>
       </c>
-      <c r="X20" t="inlineStr"/>
       <c r="Y20" t="inlineStr">
         <is>
           <t>single donor SPC2-ST-B2; paired promotion D-0014; WT-YAP is a lentiviral control, not an untransduced control; P-0001 supportive, not confirmed</t>
@@ -2755,7 +2818,6 @@
           <t>proximal_anchor</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>CA1 organoid</t>
@@ -2766,7 +2828,6 @@
           <t>10x</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>mid_GW14_16 / week_15</t>
@@ -2777,9 +2838,17 @@
           <t>Basal cells</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Basal cells</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="K2" t="n">
+        <v>11.4</v>
+      </c>
       <c r="L2" t="inlineStr">
         <is>
           <t>proximal airway-like anchor; mixed epithelial</t>
@@ -2797,7 +2866,6 @@
           <t>proximal_anchor</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>BU3 organoid</t>
@@ -2808,7 +2876,6 @@
           <t>10x</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>mid_GW14_16 / week_15</t>
@@ -2819,9 +2886,17 @@
           <t>Basal cells</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Basal cells</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="K3" t="n">
+        <v>10.9</v>
+      </c>
       <c r="L3" t="inlineStr">
         <is>
           <t>converged proximal airway-like anchor</t>
@@ -2869,9 +2944,17 @@
           <t>Tip cells</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Tip cells</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>13.3</v>
+      </c>
       <c r="L4" t="inlineStr">
         <is>
           <t>distal Tip-like; strongest donor</t>
@@ -2919,9 +3002,17 @@
           <t>Tip cells</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Tip cells</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>12.6</v>
+      </c>
       <c r="L5" t="inlineStr">
         <is>
           <t>distal Tip-like; supportive (low n=261)</t>
@@ -2969,9 +3060,17 @@
           <t>Tip cells</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Tip cells</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>13.6</v>
+      </c>
       <c r="L6" t="inlineStr">
         <is>
           <t>distal Tip-like; strongest donor</t>
@@ -3019,9 +3118,17 @@
           <t>Tip cells</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Tip cells</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>17.1</v>
+      </c>
       <c r="L7" t="inlineStr">
         <is>
           <t>distal Tip-like; consistent</t>

</xml_diff>